<commit_message>
data: update from lockring1.xlsx
- Replace old lockring.xlsx with lockring1.xlsx data
- Update excelData with 18 groups from new Excel file
- All pipe sizes and part info now reflect updated data
</commit_message>
<xml_diff>
--- a/lockring.xlsx
+++ b/lockring.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github-remote-fold-distribute-V1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDE4515E-7D97-4AD5-BC2D-04D9974E2D03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE3B93AD-4A0A-4FB5-98BA-A8D85F298758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34785" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{02909DCD-F50C-4CF1-B9FE-33B3B5C85AC8}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{02909DCD-F50C-4CF1-B9FE-33B3B5C85AC8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -758,6 +758,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F599BFA-99FB-458D-8470-E3F581F62E08}">
   <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="15.625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.25" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
@@ -1222,6 +1229,7 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Calibri"&amp;12&amp;K000000 LGE Internal Use Only&amp;1#_x000D_</oddHeader>
   </headerFooter>

</xml_diff>